<commit_message>
pull updates from https://github.com/reveron-consulting/RI_V3/commits/ray_FM/
</commit_message>
<xml_diff>
--- a/Templates/Document_Template_sslr.xlsx
+++ b/Templates/Document_Template_sslr.xlsx
@@ -1,28 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="23040" windowHeight="9000"/>
+    <workbookView windowWidth="23040" windowHeight="9024"/>
   </bookViews>
   <sheets>
     <sheet name="Doc record data" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <calcPr calcId="144525"/>
 </workbook>
 </file>
 
@@ -100,7 +87,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D1" authorId="0">
+    <comment ref="C1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -139,7 +126,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E1" authorId="0">
+    <comment ref="D1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -153,30 +140,15 @@
         </r>
         <r>
           <rPr>
-            <b/>
-            <sz val="9"/>
-            <rFont val="Tahoma"/>
-            <charset val="134"/>
-          </rPr>
-          <t>Value:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <rFont val="Tahoma"/>
-            <charset val="134"/>
-          </rPr>
-          <t xml:space="preserve">
-Construction,
-Contract Management,
-Digital Construction &amp; Asset Management,
-Health, Safety, Environment &amp; Traffic,
-Planning &amp; Scheduling,
-Quality</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="F1" authorId="0">
+            <sz val="9"/>
+            <rFont val="Tahoma"/>
+            <charset val="134"/>
+          </rPr>
+          <t>Refer to the document type setup</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="E1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -215,7 +187,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="G1" authorId="0">
+    <comment ref="F1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -245,7 +217,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="K1" authorId="0">
+    <comment ref="G1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -283,7 +255,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="M1" authorId="0">
+    <comment ref="I1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -296,7 +268,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="N1" authorId="0">
+    <comment ref="J1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -310,7 +282,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="O1" authorId="0">
+    <comment ref="K1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -339,7 +311,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="P1" authorId="0">
+    <comment ref="L1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -368,7 +340,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="Q1" authorId="0">
+    <comment ref="M1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -381,65 +353,65 @@
         </r>
       </text>
     </comment>
+    <comment ref="N1" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <rFont val="Tahoma"/>
+            <charset val="134"/>
+          </rPr>
+          <t>The average value for this record based on month. User also can edit the value once the record id uploaded.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="Q1" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">Revision is only for drawing and HSE documents. Can have values </t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <rFont val="Tahoma"/>
+            <charset val="134"/>
+          </rPr>
+          <t>Yes/No /Null</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">. IF Yes then Revison No is </t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <rFont val="Tahoma"/>
+            <charset val="134"/>
+          </rPr>
+          <t>mandatory</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <rFont val="Tahoma"/>
+            <charset val="134"/>
+          </rPr>
+          <t>.</t>
+        </r>
+      </text>
+    </comment>
     <comment ref="R1" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <rFont val="Tahoma"/>
-            <charset val="134"/>
-          </rPr>
-          <t>The average value for this record based on month. User also can edit the value once the record id uploaded.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="U1" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <rFont val="Tahoma"/>
-            <charset val="1"/>
-          </rPr>
-          <t xml:space="preserve">Revision is only for drawing and HSE documents. Can have values </t>
-        </r>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <rFont val="Tahoma"/>
-            <charset val="134"/>
-          </rPr>
-          <t>Yes/No /Null</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <rFont val="Tahoma"/>
-            <charset val="1"/>
-          </rPr>
-          <t xml:space="preserve">. IF Yes then Revison No is </t>
-        </r>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <rFont val="Tahoma"/>
-            <charset val="134"/>
-          </rPr>
-          <t>mandatory</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <rFont val="Tahoma"/>
-            <charset val="134"/>
-          </rPr>
-          <t>.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="V1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -469,7 +441,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="X1" authorId="0">
+    <comment ref="T1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -491,7 +463,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="Z1" authorId="0">
+    <comment ref="V1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -514,7 +486,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AA1" authorId="0">
+    <comment ref="W1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -536,7 +508,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AB1" authorId="0">
+    <comment ref="X1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -558,7 +530,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AC1" authorId="0">
+    <comment ref="Y1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -613,7 +585,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AD1" authorId="0">
+    <comment ref="Z1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -635,7 +607,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AE1" authorId="0">
+    <comment ref="AA1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -657,7 +629,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AF1" authorId="0">
+    <comment ref="AB1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -679,7 +651,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AH1" authorId="0">
+    <comment ref="AD1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -702,7 +674,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AI1" authorId="0">
+    <comment ref="AE1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -715,7 +687,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AJ1" authorId="0">
+    <comment ref="AF1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -742,7 +714,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="32">
   <si>
     <t>Department</t>
   </si>
@@ -750,9 +722,6 @@
     <t>Classification</t>
   </si>
   <si>
-    <t>Site Document Reference No.</t>
-  </si>
-  <si>
     <t>Section</t>
   </si>
   <si>
@@ -763,15 +732,6 @@
   </si>
   <si>
     <t>Document Sub Type</t>
-  </si>
-  <si>
-    <t>Drawing Category</t>
-  </si>
-  <si>
-    <t>Drawing Discipline</t>
-  </si>
-  <si>
-    <t>Drawing Sub-Category</t>
   </si>
   <si>
     <t>Reference No (unique)</t>
@@ -855,7 +815,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9">
   <numFmts count="4">
     <numFmt numFmtId="176" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="177" formatCode="_-&quot;RM&quot;* #,##0.00_-;\-&quot;RM&quot;* #,##0.00_-;_-&quot;RM&quot;* &quot;-&quot;??_-;_-@_-"/>
@@ -1019,12 +979,12 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
       <sz val="9"/>
       <name val="Tahoma"/>
       <charset val="1"/>
     </font>
     <font>
+      <b/>
       <sz val="9"/>
       <name val="Tahoma"/>
       <charset val="1"/>
@@ -1747,41 +1707,39 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:AJ3"/>
+  <dimension ref="A1:AF3"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" outlineLevelRow="2"/>
   <cols>
     <col min="1" max="1" width="23.8888888888889" style="1" customWidth="1"/>
-    <col min="2" max="2" width="13.6666666666667" style="1" customWidth="1"/>
-    <col min="3" max="3" width="27.7777777777778" style="1" customWidth="1"/>
-    <col min="4" max="4" width="13.6666666666667" style="1" customWidth="1"/>
-    <col min="5" max="6" width="28.3333333333333" style="1" customWidth="1"/>
-    <col min="7" max="7" width="17.3333333333333" style="1" customWidth="1"/>
-    <col min="8" max="12" width="35.7777777777778" style="1" customWidth="1"/>
-    <col min="13" max="13" width="23.6666666666667" style="1" customWidth="1"/>
-    <col min="14" max="14" width="22.6666666666667" style="1" customWidth="1"/>
-    <col min="15" max="15" width="12.5555555555556" style="1" customWidth="1"/>
-    <col min="16" max="16" width="8.88888888888889" style="1"/>
-    <col min="17" max="17" width="17.8888888888889" style="1" customWidth="1"/>
-    <col min="18" max="20" width="18.2222222222222" style="1" customWidth="1"/>
-    <col min="21" max="21" width="7.88888888888889" style="1" customWidth="1"/>
-    <col min="22" max="22" width="12.3333333333333" style="1" customWidth="1"/>
-    <col min="23" max="23" width="30.1111111111111" style="1" customWidth="1"/>
-    <col min="24" max="24" width="10.4444444444444" style="1" customWidth="1"/>
-    <col min="25" max="25" width="9.44444444444444" style="1" customWidth="1"/>
+    <col min="2" max="3" width="13.6666666666667" style="1" customWidth="1"/>
+    <col min="4" max="5" width="28.3333333333333" style="1" customWidth="1"/>
+    <col min="6" max="6" width="17.3333333333333" style="1" customWidth="1"/>
+    <col min="7" max="8" width="35.7777777777778" style="1" customWidth="1"/>
+    <col min="9" max="9" width="23.6666666666667" style="1" customWidth="1"/>
+    <col min="10" max="10" width="22.6666666666667" style="1" customWidth="1"/>
+    <col min="11" max="11" width="12.5555555555556" style="1" customWidth="1"/>
+    <col min="12" max="12" width="8.88888888888889" style="1"/>
+    <col min="13" max="13" width="17.8888888888889" style="1" customWidth="1"/>
+    <col min="14" max="16" width="18.2222222222222" style="1" customWidth="1"/>
+    <col min="17" max="17" width="7.88888888888889" style="1" customWidth="1"/>
+    <col min="18" max="18" width="12.3333333333333" style="1" customWidth="1"/>
+    <col min="19" max="19" width="30.1111111111111" style="1" customWidth="1"/>
+    <col min="20" max="20" width="10.4444444444444" style="1" customWidth="1"/>
+    <col min="21" max="21" width="9.44444444444444" style="1" customWidth="1"/>
+    <col min="22" max="22" width="14.6666666666667" style="1" customWidth="1"/>
+    <col min="23" max="23" width="18.3333333333333" style="1" customWidth="1"/>
+    <col min="24" max="25" width="8.88888888888889" style="1"/>
     <col min="26" max="26" width="14.6666666666667" style="1" customWidth="1"/>
-    <col min="27" max="27" width="18.3333333333333" style="1" customWidth="1"/>
-    <col min="28" max="29" width="8.88888888888889" style="1"/>
-    <col min="30" max="30" width="14.6666666666667" style="1" customWidth="1"/>
-    <col min="31" max="31" width="12" style="1" customWidth="1"/>
-    <col min="32" max="32" width="15.2222222222222" style="1" customWidth="1"/>
-    <col min="33" max="33" width="8.88888888888889" style="1"/>
-    <col min="34" max="34" width="17.4444444444444" style="1" customWidth="1"/>
-    <col min="35" max="35" width="22.1111111111111" style="1" customWidth="1"/>
-    <col min="36" max="36" width="26.2222222222222" style="1" customWidth="1"/>
-    <col min="37" max="16384" width="8.88888888888889" style="1"/>
+    <col min="27" max="27" width="12" style="1" customWidth="1"/>
+    <col min="28" max="28" width="15.2222222222222" style="1" customWidth="1"/>
+    <col min="29" max="29" width="8.88888888888889" style="1"/>
+    <col min="30" max="30" width="17.4444444444444" style="1" customWidth="1"/>
+    <col min="31" max="31" width="22.1111111111111" style="1" customWidth="1"/>
+    <col min="32" max="32" width="26.2222222222222" style="1" customWidth="1"/>
+    <col min="33" max="16384" width="8.88888888888889" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36">
+    <row r="1" spans="1:32">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1830,7 +1788,7 @@
       <c r="P1" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="2" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
       <c r="R1" s="2" t="s">
@@ -1839,7 +1797,7 @@
       <c r="S1" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="2" t="s">
+      <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
       <c r="U1" s="1" t="s">
@@ -1851,10 +1809,10 @@
       <c r="W1" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="X1" s="1" t="s">
+      <c r="X1" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" s="1" t="s">
+      <c r="Y1" s="2" t="s">
         <v>24</v>
       </c>
       <c r="Z1" s="2" t="s">
@@ -1878,32 +1836,20 @@
       <c r="AF1" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="AG1" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="AH1" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="AI1" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="AJ1" s="2" t="s">
-        <v>35</v>
-      </c>
     </row>
-    <row r="2" spans="26:35">
+    <row r="2" spans="22:31">
+      <c r="V2" s="3"/>
       <c r="Z2" s="3"/>
-      <c r="AD2" s="3"/>
+      <c r="AA2" s="4"/>
+      <c r="AB2" s="4"/>
       <c r="AE2" s="4"/>
-      <c r="AF2" s="4"/>
-      <c r="AI2" s="4"/>
     </row>
-    <row r="3" spans="26:35">
+    <row r="3" spans="22:31">
+      <c r="V3" s="3"/>
       <c r="Z3" s="3"/>
-      <c r="AD3" s="3"/>
+      <c r="AA3" s="4"/>
+      <c r="AB3" s="4"/>
       <c r="AE3" s="4"/>
-      <c r="AF3" s="4"/>
-      <c r="AI3" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
pull updates fromo https://github.com/reveron-consulting/RI_V3/commits/reveronInsights/
</commit_message>
<xml_diff>
--- a/Templates/Document_Template_sslr.xlsx
+++ b/Templates/Document_Template_sslr.xlsx
@@ -1,15 +1,28 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="23040" windowHeight="9024"/>
+    <workbookView windowWidth="23040" windowHeight="9000"/>
   </bookViews>
   <sheets>
     <sheet name="Doc record data" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="144525"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -87,7 +100,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C1" authorId="0">
+    <comment ref="D1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -126,7 +139,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D1" authorId="0">
+    <comment ref="E1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -140,15 +153,30 @@
         </r>
         <r>
           <rPr>
-            <sz val="9"/>
-            <rFont val="Tahoma"/>
-            <charset val="134"/>
-          </rPr>
-          <t>Refer to the document type setup</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="E1" authorId="0">
+            <b/>
+            <sz val="9"/>
+            <rFont val="Tahoma"/>
+            <charset val="134"/>
+          </rPr>
+          <t>Value:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <rFont val="Tahoma"/>
+            <charset val="134"/>
+          </rPr>
+          <t xml:space="preserve">
+Construction,
+Contract Management,
+Digital Construction &amp; Asset Management,
+Health, Safety, Environment &amp; Traffic,
+Planning &amp; Scheduling,
+Quality</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="F1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -187,7 +215,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="F1" authorId="0">
+    <comment ref="G1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -217,7 +245,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="G1" authorId="0">
+    <comment ref="K1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -255,7 +283,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="I1" authorId="0">
+    <comment ref="M1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -268,7 +296,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="J1" authorId="0">
+    <comment ref="N1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -282,7 +310,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="K1" authorId="0">
+    <comment ref="O1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -311,7 +339,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="L1" authorId="0">
+    <comment ref="P1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -340,7 +368,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="M1" authorId="0">
+    <comment ref="Q1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -353,7 +381,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="N1" authorId="0">
+    <comment ref="R1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -365,7 +393,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="Q1" authorId="0">
+    <comment ref="U1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -411,7 +439,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="R1" authorId="0">
+    <comment ref="V1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -441,7 +469,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="T1" authorId="0">
+    <comment ref="X1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -463,7 +491,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="V1" authorId="0">
+    <comment ref="Z1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -486,7 +514,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="W1" authorId="0">
+    <comment ref="AA1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -508,7 +536,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="X1" authorId="0">
+    <comment ref="AB1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -530,7 +558,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="Y1" authorId="0">
+    <comment ref="AC1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -585,7 +613,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="Z1" authorId="0">
+    <comment ref="AD1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -607,7 +635,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AA1" authorId="0">
+    <comment ref="AE1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -629,7 +657,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AB1" authorId="0">
+    <comment ref="AF1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -651,7 +679,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AD1" authorId="0">
+    <comment ref="AH1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -674,7 +702,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AE1" authorId="0">
+    <comment ref="AI1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -687,7 +715,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AF1" authorId="0">
+    <comment ref="AJ1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -714,7 +742,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="36">
   <si>
     <t>Department</t>
   </si>
@@ -722,6 +750,9 @@
     <t>Classification</t>
   </si>
   <si>
+    <t>Site Document Reference No.</t>
+  </si>
+  <si>
     <t>Section</t>
   </si>
   <si>
@@ -732,6 +763,15 @@
   </si>
   <si>
     <t>Document Sub Type</t>
+  </si>
+  <si>
+    <t>Drawing Category</t>
+  </si>
+  <si>
+    <t>Drawing Discipline</t>
+  </si>
+  <si>
+    <t>Drawing Sub-Category</t>
   </si>
   <si>
     <t>Reference No (unique)</t>
@@ -815,7 +855,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
   <numFmts count="4">
     <numFmt numFmtId="176" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="177" formatCode="_-&quot;RM&quot;* #,##0.00_-;\-&quot;RM&quot;* #,##0.00_-;_-&quot;RM&quot;* &quot;-&quot;??_-;_-@_-"/>
@@ -979,12 +1019,12 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
       <sz val="9"/>
       <name val="Tahoma"/>
       <charset val="1"/>
     </font>
     <font>
-      <b/>
       <sz val="9"/>
       <name val="Tahoma"/>
       <charset val="1"/>
@@ -1707,39 +1747,41 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:AF3"/>
+  <dimension ref="A1:AJ3"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" outlineLevelRow="2"/>
   <cols>
     <col min="1" max="1" width="23.8888888888889" style="1" customWidth="1"/>
-    <col min="2" max="3" width="13.6666666666667" style="1" customWidth="1"/>
-    <col min="4" max="5" width="28.3333333333333" style="1" customWidth="1"/>
-    <col min="6" max="6" width="17.3333333333333" style="1" customWidth="1"/>
-    <col min="7" max="8" width="35.7777777777778" style="1" customWidth="1"/>
-    <col min="9" max="9" width="23.6666666666667" style="1" customWidth="1"/>
-    <col min="10" max="10" width="22.6666666666667" style="1" customWidth="1"/>
-    <col min="11" max="11" width="12.5555555555556" style="1" customWidth="1"/>
-    <col min="12" max="12" width="8.88888888888889" style="1"/>
-    <col min="13" max="13" width="17.8888888888889" style="1" customWidth="1"/>
-    <col min="14" max="16" width="18.2222222222222" style="1" customWidth="1"/>
-    <col min="17" max="17" width="7.88888888888889" style="1" customWidth="1"/>
-    <col min="18" max="18" width="12.3333333333333" style="1" customWidth="1"/>
-    <col min="19" max="19" width="30.1111111111111" style="1" customWidth="1"/>
-    <col min="20" max="20" width="10.4444444444444" style="1" customWidth="1"/>
-    <col min="21" max="21" width="9.44444444444444" style="1" customWidth="1"/>
-    <col min="22" max="22" width="14.6666666666667" style="1" customWidth="1"/>
-    <col min="23" max="23" width="18.3333333333333" style="1" customWidth="1"/>
-    <col min="24" max="25" width="8.88888888888889" style="1"/>
+    <col min="2" max="2" width="13.6666666666667" style="1" customWidth="1"/>
+    <col min="3" max="3" width="27.7777777777778" style="1" customWidth="1"/>
+    <col min="4" max="4" width="13.6666666666667" style="1" customWidth="1"/>
+    <col min="5" max="6" width="28.3333333333333" style="1" customWidth="1"/>
+    <col min="7" max="7" width="17.3333333333333" style="1" customWidth="1"/>
+    <col min="8" max="12" width="35.7777777777778" style="1" customWidth="1"/>
+    <col min="13" max="13" width="23.6666666666667" style="1" customWidth="1"/>
+    <col min="14" max="14" width="22.6666666666667" style="1" customWidth="1"/>
+    <col min="15" max="15" width="12.5555555555556" style="1" customWidth="1"/>
+    <col min="16" max="16" width="8.88888888888889" style="1"/>
+    <col min="17" max="17" width="17.8888888888889" style="1" customWidth="1"/>
+    <col min="18" max="20" width="18.2222222222222" style="1" customWidth="1"/>
+    <col min="21" max="21" width="7.88888888888889" style="1" customWidth="1"/>
+    <col min="22" max="22" width="12.3333333333333" style="1" customWidth="1"/>
+    <col min="23" max="23" width="30.1111111111111" style="1" customWidth="1"/>
+    <col min="24" max="24" width="10.4444444444444" style="1" customWidth="1"/>
+    <col min="25" max="25" width="9.44444444444444" style="1" customWidth="1"/>
     <col min="26" max="26" width="14.6666666666667" style="1" customWidth="1"/>
-    <col min="27" max="27" width="12" style="1" customWidth="1"/>
-    <col min="28" max="28" width="15.2222222222222" style="1" customWidth="1"/>
-    <col min="29" max="29" width="8.88888888888889" style="1"/>
-    <col min="30" max="30" width="17.4444444444444" style="1" customWidth="1"/>
-    <col min="31" max="31" width="22.1111111111111" style="1" customWidth="1"/>
-    <col min="32" max="32" width="26.2222222222222" style="1" customWidth="1"/>
-    <col min="33" max="16384" width="8.88888888888889" style="1"/>
+    <col min="27" max="27" width="18.3333333333333" style="1" customWidth="1"/>
+    <col min="28" max="29" width="8.88888888888889" style="1"/>
+    <col min="30" max="30" width="14.6666666666667" style="1" customWidth="1"/>
+    <col min="31" max="31" width="12" style="1" customWidth="1"/>
+    <col min="32" max="32" width="15.2222222222222" style="1" customWidth="1"/>
+    <col min="33" max="33" width="8.88888888888889" style="1"/>
+    <col min="34" max="34" width="17.4444444444444" style="1" customWidth="1"/>
+    <col min="35" max="35" width="22.1111111111111" style="1" customWidth="1"/>
+    <col min="36" max="36" width="26.2222222222222" style="1" customWidth="1"/>
+    <col min="37" max="16384" width="8.88888888888889" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:32">
+    <row r="1" spans="1:36">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1788,7 +1830,7 @@
       <c r="P1" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" s="2" t="s">
         <v>16</v>
       </c>
       <c r="R1" s="2" t="s">
@@ -1797,7 +1839,7 @@
       <c r="S1" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" s="2" t="s">
         <v>19</v>
       </c>
       <c r="U1" s="1" t="s">
@@ -1809,10 +1851,10 @@
       <c r="W1" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="X1" s="2" t="s">
+      <c r="X1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" s="2" t="s">
+      <c r="Y1" s="1" t="s">
         <v>24</v>
       </c>
       <c r="Z1" s="2" t="s">
@@ -1836,20 +1878,32 @@
       <c r="AF1" s="2" t="s">
         <v>31</v>
       </c>
+      <c r="AG1" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="AH1" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="AI1" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="AJ1" s="2" t="s">
+        <v>35</v>
+      </c>
     </row>
-    <row r="2" spans="22:31">
-      <c r="V2" s="3"/>
+    <row r="2" spans="26:35">
       <c r="Z2" s="3"/>
-      <c r="AA2" s="4"/>
-      <c r="AB2" s="4"/>
+      <c r="AD2" s="3"/>
       <c r="AE2" s="4"/>
+      <c r="AF2" s="4"/>
+      <c r="AI2" s="4"/>
     </row>
-    <row r="3" spans="22:31">
-      <c r="V3" s="3"/>
+    <row r="3" spans="26:35">
       <c r="Z3" s="3"/>
-      <c r="AA3" s="4"/>
-      <c r="AB3" s="4"/>
+      <c r="AD3" s="3"/>
       <c r="AE3" s="4"/>
+      <c r="AF3" s="4"/>
+      <c r="AI3" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>